<commit_message>
implement window energy baseline and add results file
</commit_message>
<xml_diff>
--- a/baselines/threshold-based-baseline/predicted_X_df_baseline.xlsx
+++ b/baselines/threshold-based-baseline/predicted_X_df_baseline.xlsx
@@ -446,7 +446,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -456,7 +456,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -466,7 +466,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -506,7 +506,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -516,7 +516,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -566,7 +566,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -586,7 +586,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -606,7 +606,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -756,7 +756,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -786,7 +786,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -796,7 +796,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -806,7 +806,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -816,7 +816,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -896,7 +896,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -1886,7 +1886,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -1896,7 +1896,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -1906,7 +1906,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -1926,7 +1926,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -1936,7 +1936,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -1946,7 +1946,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -1976,7 +1976,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -1996,7 +1996,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -2026,7 +2026,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -2166,7 +2166,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -2176,7 +2176,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -2196,7 +2196,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -2216,7 +2216,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -2226,7 +2226,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -2236,7 +2236,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -2246,7 +2246,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -2256,7 +2256,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -2266,7 +2266,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -2286,7 +2286,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2296,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -2306,7 +2306,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -2336,7 +2336,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -2346,7 +2346,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2356,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -2366,7 +2366,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -2376,7 +2376,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -2386,7 +2386,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -2456,7 +2456,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -2466,7 +2466,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -2516,7 +2516,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -2526,7 +2526,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -2536,7 +2536,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -2546,7 +2546,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -2556,7 +2556,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -2666,7 +2666,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -2686,7 +2686,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -2696,7 +2696,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -2706,7 +2706,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -2716,7 +2716,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -2726,7 +2726,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -2746,7 +2746,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -2776,7 +2776,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -2816,7 +2816,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -2826,7 +2826,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -2836,7 +2836,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -2886,7 +2886,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -2896,7 +2896,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -2906,7 +2906,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -2916,7 +2916,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -2926,7 +2926,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -2936,7 +2936,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -2956,7 +2956,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -2966,7 +2966,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -2986,7 +2986,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -3006,7 +3006,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -3036,7 +3036,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -3046,7 +3046,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -3056,7 +3056,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -3066,7 +3066,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -3096,7 +3096,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -3106,7 +3106,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3116,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -3126,7 +3126,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -3136,7 +3136,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -3146,7 +3146,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -3156,7 +3156,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -3166,7 +3166,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -3236,7 +3236,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -3246,7 +3246,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -3256,7 +3256,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -3266,7 +3266,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -3276,7 +3276,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -3286,7 +3286,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -3326,7 +3326,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -3336,7 +3336,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -3346,7 +3346,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -3416,7 +3416,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -3426,7 +3426,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -3436,7 +3436,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -3456,7 +3456,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -3466,7 +3466,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -3476,7 +3476,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -3486,7 +3486,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -3506,7 +3506,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -3536,7 +3536,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -3546,7 +3546,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -3556,7 +3556,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -3586,7 +3586,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -3596,7 +3596,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -3606,7 +3606,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -3626,7 +3626,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -3646,7 +3646,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -3656,7 +3656,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -3666,7 +3666,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -3676,7 +3676,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -3696,7 +3696,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -3706,7 +3706,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -3716,7 +3716,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -3726,7 +3726,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
@@ -3736,7 +3736,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
@@ -3756,7 +3756,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
@@ -3766,7 +3766,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>eID_3</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>

</xml_diff>